<commit_message>
HANDOFF·WBS 갱신: 실제 Claude 연결 준비(PR #20)
</commit_message>
<xml_diff>
--- a/docs/WBS.xlsx
+++ b/docs/WBS.xlsx
@@ -2019,18 +2019,34 @@
           <t>개발</t>
         </is>
       </c>
-      <c r="F36" s="16" t="n"/>
-      <c r="G36" s="16" t="n"/>
+      <c r="F36" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="G36" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
       <c r="H36" s="16" t="inlineStr">
         <is>
-          <t>예정</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="I36" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J36" s="8" t="n"/>
-      <c r="K36" s="8" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="J36" s="8" t="inlineStr">
+        <is>
+          <t>PR #20</t>
+        </is>
+      </c>
+      <c r="K36" s="8" t="inlineStr">
+        <is>
+          <t>어댑터 준비(기본 Mock). 실제 호출·모델·비용은 인수 기업</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="16" t="inlineStr">

</xml_diff>

<commit_message>
실제 Claude 연결 준비(ClaudeProvider, 기본은 Mock·비용 0) (#20)
* 실제 Claude 연결 계획

* 실제 Claude 연결: ClaudeProvider(공식 SDK, 구조화 출력·캐시·거절 대체), PROVIDER=claude 설정과 확인 스크립트

* 리뷰 수정(Claude): 거절·잘림을 검증 전에 판정(create+json_schema), 키 없으면 시작 때 알림, Haiku는 대체 모델 없이

* HANDOFF·WBS 갱신: 실제 Claude 연결 준비(PR #20)
</commit_message>
<xml_diff>
--- a/docs/WBS.xlsx
+++ b/docs/WBS.xlsx
@@ -2019,18 +2019,34 @@
           <t>개발</t>
         </is>
       </c>
-      <c r="F36" s="16" t="n"/>
-      <c r="G36" s="16" t="n"/>
+      <c r="F36" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="G36" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
       <c r="H36" s="16" t="inlineStr">
         <is>
-          <t>예정</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="I36" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J36" s="8" t="n"/>
-      <c r="K36" s="8" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="J36" s="8" t="inlineStr">
+        <is>
+          <t>PR #20</t>
+        </is>
+      </c>
+      <c r="K36" s="8" t="inlineStr">
+        <is>
+          <t>어댑터 준비(기본 Mock). 실제 호출·모델·비용은 인수 기업</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="16" t="inlineStr">

</xml_diff>

<commit_message>
문서: 외부 전송 보호(README, HANDOFF 한계, CLAUDE.md 원칙, WBS 6.4)
</commit_message>
<xml_diff>
--- a/docs/WBS.xlsx
+++ b/docs/WBS.xlsx
@@ -11,7 +11,7 @@
     <sheet name="요약" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WBS'!$A$4:$K$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WBS'!$A$4:$K$43</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -98,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -129,6 +129,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -529,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -645,12 +651,12 @@
       <c r="K5" s="5" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>1.1</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>기획·설계</t>
         </is>
@@ -665,23 +671,23 @@
           <t>과제 4개(사업계획·상품기획·브랜딩·마케팅), 적응형 질문, 사실·가정 분리 원칙</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E6" s="20" t="inlineStr">
         <is>
           <t>공동</t>
         </is>
       </c>
-      <c r="F6" s="16" t="n"/>
-      <c r="G6" s="16" t="inlineStr">
+      <c r="F6" s="20" t="n"/>
+      <c r="G6" s="20" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="H6" s="16" t="inlineStr">
+      <c r="H6" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I6" s="17" t="n">
+      <c r="I6" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J6" s="8" t="inlineStr">
@@ -692,12 +698,12 @@
       <c r="K6" s="8" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>기획·설계</t>
         </is>
@@ -712,27 +718,27 @@
           <t>FastAPI 하네스 구조, API 계약, 테스트 전략</t>
         </is>
       </c>
-      <c r="E7" s="16" t="inlineStr">
+      <c r="E7" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F7" s="16" t="inlineStr">
+      <c r="F7" s="20" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="G7" s="20" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I7" s="17" t="n">
+      <c r="I7" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J7" s="8" t="inlineStr">
@@ -743,12 +749,12 @@
       <c r="K7" s="8" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>1.3</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>기획·설계</t>
         </is>
@@ -763,27 +769,27 @@
           <t>V2 화면 흐름, 묶음 0~4로 작업 나누기</t>
         </is>
       </c>
-      <c r="E8" s="16" t="inlineStr">
+      <c r="E8" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F8" s="16" t="inlineStr">
+      <c r="F8" s="20" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G8" s="16" t="inlineStr">
+      <c r="G8" s="20" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H8" s="16" t="inlineStr">
+      <c r="H8" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I8" s="17" t="n">
+      <c r="I8" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J8" s="8" t="inlineStr">
@@ -794,12 +800,12 @@
       <c r="K8" s="8" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>기획·설계</t>
         </is>
@@ -814,27 +820,27 @@
           <t>지금 상태·다음 할 일·작업 방식·환경 팁, PR마다 갱신</t>
         </is>
       </c>
-      <c r="E9" s="16" t="inlineStr">
+      <c r="E9" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F9" s="16" t="inlineStr">
+      <c r="F9" s="20" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="G9" s="16" t="inlineStr">
+      <c r="G9" s="20" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="H9" s="16" t="inlineStr">
+      <c r="H9" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I9" s="17" t="n">
+      <c r="I9" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J9" s="8" t="inlineStr">
@@ -845,12 +851,12 @@
       <c r="K9" s="8" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>기획·설계</t>
         </is>
@@ -865,27 +871,27 @@
           <t>바로 보기 주소, 된 것, 남은 일·맡을 사람·상의할 점</t>
         </is>
       </c>
-      <c r="E10" s="18" t="inlineStr">
+      <c r="E10" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="F10" s="20" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="G10" s="18" t="inlineStr">
+      <c r="G10" s="20" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="H10" s="18" t="inlineStr">
+      <c r="H10" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I10" s="19" t="n">
+      <c r="I10" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J10" s="8" t="inlineStr">
@@ -924,12 +930,12 @@
       <c r="K11" s="5" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>2.1</t>
         </is>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>백엔드 기반</t>
         </is>
@@ -944,27 +950,27 @@
           <t>사실·가정·미정 구분, 정보 출처 표시</t>
         </is>
       </c>
-      <c r="E12" s="16" t="inlineStr">
+      <c r="E12" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F12" s="16" t="inlineStr">
+      <c r="F12" s="20" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G12" s="16" t="inlineStr">
+      <c r="G12" s="20" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H12" s="16" t="inlineStr">
+      <c r="H12" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I12" s="17" t="n">
+      <c r="I12" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J12" s="8" t="inlineStr">
@@ -975,12 +981,12 @@
       <c r="K12" s="8" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>백엔드 기반</t>
         </is>
@@ -995,27 +1001,27 @@
           <t>비용 없이 개발·테스트하는 가짜 모델</t>
         </is>
       </c>
-      <c r="E13" s="16" t="inlineStr">
+      <c r="E13" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F13" s="16" t="inlineStr">
+      <c r="F13" s="20" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G13" s="16" t="inlineStr">
+      <c r="G13" s="20" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H13" s="16" t="inlineStr">
+      <c r="H13" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I13" s="17" t="n">
+      <c r="I13" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J13" s="8" t="inlineStr">
@@ -1026,12 +1032,12 @@
       <c r="K13" s="8" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="20" t="inlineStr">
         <is>
           <t>백엔드 기반</t>
         </is>
@@ -1046,27 +1052,27 @@
           <t>과제별 질문 정책(policy.yaml), 단계별 프롬프트</t>
         </is>
       </c>
-      <c r="E14" s="16" t="inlineStr">
+      <c r="E14" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F14" s="16" t="inlineStr">
+      <c r="F14" s="20" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G14" s="16" t="inlineStr">
+      <c r="G14" s="20" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H14" s="16" t="inlineStr">
+      <c r="H14" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I14" s="17" t="n">
+      <c r="I14" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J14" s="8" t="inlineStr">
@@ -1077,12 +1083,12 @@
       <c r="K14" s="8" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="20" t="inlineStr">
         <is>
           <t>백엔드 기반</t>
         </is>
@@ -1097,27 +1103,27 @@
           <t>모드별 질문 상한, '다른 예시 보기' 단계</t>
         </is>
       </c>
-      <c r="E15" s="16" t="inlineStr">
+      <c r="E15" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F15" s="16" t="inlineStr">
+      <c r="F15" s="20" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G15" s="16" t="inlineStr">
+      <c r="G15" s="20" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H15" s="16" t="inlineStr">
+      <c r="H15" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I15" s="17" t="n">
+      <c r="I15" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J15" s="8" t="inlineStr">
@@ -1128,12 +1134,12 @@
       <c r="K15" s="8" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>2.5</t>
         </is>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="20" t="inlineStr">
         <is>
           <t>백엔드 기반</t>
         </is>
@@ -1144,27 +1150,27 @@
         </is>
       </c>
       <c r="D16" s="8" t="n"/>
-      <c r="E16" s="16" t="inlineStr">
+      <c r="E16" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F16" s="16" t="inlineStr">
+      <c r="F16" s="20" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G16" s="16" t="inlineStr">
+      <c r="G16" s="20" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H16" s="16" t="inlineStr">
+      <c r="H16" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I16" s="17" t="n">
+      <c r="I16" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J16" s="8" t="inlineStr">
@@ -1175,12 +1181,12 @@
       <c r="K16" s="8" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="20" t="inlineStr">
         <is>
           <t>백엔드 기반</t>
         </is>
@@ -1195,27 +1201,27 @@
           <t>과제별 정책·프롬프트·검증 규칙</t>
         </is>
       </c>
-      <c r="E17" s="16" t="inlineStr">
+      <c r="E17" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F17" s="16" t="inlineStr">
+      <c r="F17" s="20" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G17" s="16" t="inlineStr">
+      <c r="G17" s="20" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H17" s="16" t="inlineStr">
+      <c r="H17" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I17" s="17" t="n">
+      <c r="I17" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J17" s="8" t="inlineStr">
@@ -1226,12 +1232,12 @@
       <c r="K17" s="8" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>2.7</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="20" t="inlineStr">
         <is>
           <t>백엔드 기반</t>
         </is>
@@ -1246,27 +1252,27 @@
           <t>한국어 오류 문구, API 문서</t>
         </is>
       </c>
-      <c r="E18" s="16" t="inlineStr">
+      <c r="E18" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F18" s="16" t="inlineStr">
+      <c r="F18" s="20" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G18" s="16" t="inlineStr">
+      <c r="G18" s="20" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H18" s="16" t="inlineStr">
+      <c r="H18" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I18" s="17" t="n">
+      <c r="I18" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J18" s="8" t="inlineStr">
@@ -1277,12 +1283,12 @@
       <c r="K18" s="8" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>2.8</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="20" t="inlineStr">
         <is>
           <t>백엔드 기반</t>
         </is>
@@ -1297,27 +1303,27 @@
           <t>API에 맞춘 최소 화면, 개발 안내(CLAUDE.md)</t>
         </is>
       </c>
-      <c r="E19" s="16" t="inlineStr">
+      <c r="E19" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F19" s="16" t="inlineStr">
+      <c r="F19" s="20" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G19" s="16" t="inlineStr">
+      <c r="G19" s="20" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H19" s="16" t="inlineStr">
+      <c r="H19" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I19" s="17" t="n">
+      <c r="I19" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J19" s="8" t="inlineStr">
@@ -1356,12 +1362,12 @@
       <c r="K20" s="5" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="20" t="inlineStr">
         <is>
           <t>3.1</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="20" t="inlineStr">
         <is>
           <t>디자인</t>
         </is>
@@ -1376,23 +1382,23 @@
           <t>전체 화면 흐름 HTML 프로토타입</t>
         </is>
       </c>
-      <c r="E21" s="16" t="inlineStr">
+      <c r="E21" s="20" t="inlineStr">
         <is>
           <t>디자인</t>
         </is>
       </c>
-      <c r="F21" s="16" t="n"/>
-      <c r="G21" s="16" t="inlineStr">
+      <c r="F21" s="20" t="n"/>
+      <c r="G21" s="20" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H21" s="16" t="inlineStr">
+      <c r="H21" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I21" s="17" t="n">
+      <c r="I21" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J21" s="8" t="inlineStr">
@@ -1403,12 +1409,12 @@
       <c r="K21" s="8" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="20" t="inlineStr">
         <is>
           <t>디자인</t>
         </is>
@@ -1423,27 +1429,27 @@
           <t>모든 질문에 '다른 예시 보기', 모드 설명, 이미지 블록, 생성 중·실패·최신 아님 상태</t>
         </is>
       </c>
-      <c r="E22" s="16" t="inlineStr">
+      <c r="E22" s="20" t="inlineStr">
         <is>
           <t>디자인</t>
         </is>
       </c>
-      <c r="F22" s="16" t="inlineStr">
+      <c r="F22" s="20" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="G22" s="16" t="inlineStr">
+      <c r="G22" s="20" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="H22" s="16" t="inlineStr">
+      <c r="H22" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I22" s="17" t="n">
+      <c r="I22" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J22" s="8" t="inlineStr">
@@ -1454,12 +1460,12 @@
       <c r="K22" s="8" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="20" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
       </c>
-      <c r="B23" s="16" t="inlineStr">
+      <c r="B23" s="20" t="inlineStr">
         <is>
           <t>디자인</t>
         </is>
@@ -1474,31 +1480,31 @@
           <t>반응형 자동 배치 확인</t>
         </is>
       </c>
-      <c r="E23" s="16" t="inlineStr">
+      <c r="E23" s="20" t="inlineStr">
         <is>
           <t>디자인</t>
         </is>
       </c>
-      <c r="F23" s="16" t="n"/>
-      <c r="G23" s="16" t="n"/>
-      <c r="H23" s="16" t="inlineStr">
+      <c r="F23" s="20" t="n"/>
+      <c r="G23" s="20" t="n"/>
+      <c r="H23" s="20" t="inlineStr">
         <is>
           <t>예정</t>
         </is>
       </c>
-      <c r="I23" s="17" t="n">
+      <c r="I23" s="21" t="n">
         <v>0</v>
       </c>
       <c r="J23" s="8" t="n"/>
       <c r="K23" s="8" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="A24" s="20" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>
       </c>
-      <c r="B24" s="16" t="inlineStr">
+      <c r="B24" s="20" t="inlineStr">
         <is>
           <t>디자인</t>
         </is>
@@ -1513,19 +1519,19 @@
           <t>/preview 화면을 html.to.design으로 가져와 수정</t>
         </is>
       </c>
-      <c r="E24" s="16" t="inlineStr">
+      <c r="E24" s="20" t="inlineStr">
         <is>
           <t>디자인</t>
         </is>
       </c>
-      <c r="F24" s="16" t="n"/>
-      <c r="G24" s="16" t="n"/>
-      <c r="H24" s="16" t="inlineStr">
+      <c r="F24" s="20" t="n"/>
+      <c r="G24" s="20" t="n"/>
+      <c r="H24" s="20" t="inlineStr">
         <is>
           <t>예정</t>
         </is>
       </c>
-      <c r="I24" s="17" t="n">
+      <c r="I24" s="21" t="n">
         <v>0</v>
       </c>
       <c r="J24" s="8" t="n"/>
@@ -1560,12 +1566,12 @@
       <c r="K25" s="5" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="20" t="inlineStr">
         <is>
           <t>4.1</t>
         </is>
       </c>
-      <c r="B26" s="16" t="inlineStr">
+      <c r="B26" s="20" t="inlineStr">
         <is>
           <t>화면 개발(V2)</t>
         </is>
@@ -1580,27 +1586,27 @@
           <t>버셀 배포 설정 포함</t>
         </is>
       </c>
-      <c r="E26" s="16" t="inlineStr">
+      <c r="E26" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F26" s="16" t="inlineStr">
+      <c r="F26" s="20" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G26" s="16" t="inlineStr">
+      <c r="G26" s="20" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H26" s="16" t="inlineStr">
+      <c r="H26" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I26" s="17" t="n">
+      <c r="I26" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J26" s="8" t="inlineStr">
@@ -1611,12 +1617,12 @@
       <c r="K26" s="8" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr">
+      <c r="A27" s="20" t="inlineStr">
         <is>
           <t>4.2</t>
         </is>
       </c>
-      <c r="B27" s="16" t="inlineStr">
+      <c r="B27" s="20" t="inlineStr">
         <is>
           <t>화면 개발(V2)</t>
         </is>
@@ -1631,27 +1637,27 @@
           <t>답변 종류, 흐름 패널, 익명 사용자</t>
         </is>
       </c>
-      <c r="E27" s="16" t="inlineStr">
+      <c r="E27" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F27" s="16" t="inlineStr">
+      <c r="F27" s="20" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="G27" s="16" t="inlineStr">
+      <c r="G27" s="20" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="H27" s="16" t="inlineStr">
+      <c r="H27" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I27" s="17" t="n">
+      <c r="I27" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J27" s="8" t="inlineStr">
@@ -1662,12 +1668,12 @@
       <c r="K27" s="8" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
+      <c r="A28" s="20" t="inlineStr">
         <is>
           <t>4.3</t>
         </is>
       </c>
-      <c r="B28" s="16" t="inlineStr">
+      <c r="B28" s="20" t="inlineStr">
         <is>
           <t>화면 개발(V2)</t>
         </is>
@@ -1682,27 +1688,27 @@
           <t>서버 저장(SQLite), 문서 내려받기</t>
         </is>
       </c>
-      <c r="E28" s="16" t="inlineStr">
+      <c r="E28" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F28" s="16" t="inlineStr">
+      <c r="F28" s="20" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="G28" s="16" t="inlineStr">
+      <c r="G28" s="20" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="H28" s="16" t="inlineStr">
+      <c r="H28" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I28" s="17" t="n">
+      <c r="I28" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J28" s="8" t="inlineStr">
@@ -1713,12 +1719,12 @@
       <c r="K28" s="8" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="inlineStr">
+      <c r="A29" s="20" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
       </c>
-      <c r="B29" s="16" t="inlineStr">
+      <c r="B29" s="20" t="inlineStr">
         <is>
           <t>화면 개발(V2)</t>
         </is>
@@ -1733,27 +1739,27 @@
           <t>결과를 섹션·블록으로</t>
         </is>
       </c>
-      <c r="E29" s="16" t="inlineStr">
+      <c r="E29" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F29" s="16" t="inlineStr">
+      <c r="F29" s="20" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="G29" s="16" t="inlineStr">
+      <c r="G29" s="20" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="H29" s="16" t="inlineStr">
+      <c r="H29" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I29" s="17" t="n">
+      <c r="I29" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J29" s="8" t="inlineStr">
@@ -1764,12 +1770,12 @@
       <c r="K29" s="8" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="16" t="inlineStr">
+      <c r="A30" s="20" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="B30" s="16" t="inlineStr">
+      <c r="B30" s="20" t="inlineStr">
         <is>
           <t>화면 개발(V2)</t>
         </is>
@@ -1784,27 +1790,27 @@
           <t>샘플 근거 자료, 자리표시 이미지</t>
         </is>
       </c>
-      <c r="E30" s="16" t="inlineStr">
+      <c r="E30" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F30" s="16" t="inlineStr">
+      <c r="F30" s="20" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="G30" s="16" t="inlineStr">
+      <c r="G30" s="20" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="H30" s="16" t="inlineStr">
+      <c r="H30" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I30" s="17" t="n">
+      <c r="I30" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J30" s="8" t="inlineStr">
@@ -1815,12 +1821,12 @@
       <c r="K30" s="8" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="inlineStr">
+      <c r="A31" s="20" t="inlineStr">
         <is>
           <t>4.6</t>
         </is>
       </c>
-      <c r="B31" s="16" t="inlineStr">
+      <c r="B31" s="20" t="inlineStr">
         <is>
           <t>화면 개발(V2)</t>
         </is>
@@ -1835,27 +1841,27 @@
           <t>생성 중·생성 실패 화면, 최신 아님 배너, 이미지 상자, 모드 설명</t>
         </is>
       </c>
-      <c r="E31" s="16" t="inlineStr">
+      <c r="E31" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F31" s="16" t="inlineStr">
+      <c r="F31" s="20" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="G31" s="16" t="inlineStr">
+      <c r="G31" s="20" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="H31" s="16" t="inlineStr">
+      <c r="H31" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I31" s="17" t="n">
+      <c r="I31" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J31" s="8" t="inlineStr">
@@ -1866,12 +1872,12 @@
       <c r="K31" s="8" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="16" t="inlineStr">
+      <c r="A32" s="20" t="inlineStr">
         <is>
           <t>4.7</t>
         </is>
       </c>
-      <c r="B32" s="16" t="inlineStr">
+      <c r="B32" s="20" t="inlineStr">
         <is>
           <t>화면 개발(V2)</t>
         </is>
@@ -1886,27 +1892,27 @@
           <t>이전 결과를 다음 과제의 기준으로 가져오기</t>
         </is>
       </c>
-      <c r="E32" s="16" t="inlineStr">
+      <c r="E32" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F32" s="16" t="inlineStr">
+      <c r="F32" s="20" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="G32" s="16" t="inlineStr">
+      <c r="G32" s="20" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="H32" s="16" t="inlineStr">
+      <c r="H32" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I32" s="17" t="n">
+      <c r="I32" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J32" s="8" t="inlineStr">
@@ -1945,12 +1951,12 @@
       <c r="K33" s="5" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr">
+      <c r="A34" s="20" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
       </c>
-      <c r="B34" s="16" t="inlineStr">
+      <c r="B34" s="20" t="inlineStr">
         <is>
           <t>배포</t>
         </is>
@@ -1965,27 +1971,27 @@
           <t>main은 정식 주소, PR마다 미리보기 주소</t>
         </is>
       </c>
-      <c r="E34" s="16" t="inlineStr">
+      <c r="E34" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F34" s="16" t="inlineStr">
+      <c r="F34" s="20" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="G34" s="16" t="inlineStr">
+      <c r="G34" s="20" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="H34" s="16" t="inlineStr">
+      <c r="H34" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I34" s="17" t="n">
+      <c r="I34" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J34" s="8" t="inlineStr">
@@ -2000,12 +2006,12 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr">
+      <c r="A35" s="20" t="inlineStr">
         <is>
           <t>5.2</t>
         </is>
       </c>
-      <c r="B35" s="16" t="inlineStr">
+      <c r="B35" s="20" t="inlineStr">
         <is>
           <t>배포</t>
         </is>
@@ -2020,27 +2026,27 @@
           <t>저장 디스크 방식 정하기, 프론트와 연결</t>
         </is>
       </c>
-      <c r="E35" s="16" t="inlineStr">
+      <c r="E35" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F35" s="16" t="inlineStr">
+      <c r="F35" s="20" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="G35" s="16" t="inlineStr">
+      <c r="G35" s="20" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="H35" s="16" t="inlineStr">
+      <c r="H35" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I35" s="17" t="n">
+      <c r="I35" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J35" s="8" t="inlineStr">
@@ -2076,19 +2082,19 @@
       <c r="G36" s="4" t="n"/>
       <c r="H36" s="4" t="n"/>
       <c r="I36" s="6">
-        <f>IFERROR(AVERAGE(I37:I39),0)</f>
+        <f>IFERROR(AVERAGE(I37:I40),0)</f>
         <v/>
       </c>
       <c r="J36" s="5" t="n"/>
       <c r="K36" s="5" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="16" t="inlineStr">
+      <c r="A37" s="20" t="inlineStr">
         <is>
           <t>6.1</t>
         </is>
       </c>
-      <c r="B37" s="16" t="inlineStr">
+      <c r="B37" s="20" t="inlineStr">
         <is>
           <t>실제 AI 연결</t>
         </is>
@@ -2103,27 +2109,27 @@
           <t>가짜 모델(Mock) 대신 실제 모델</t>
         </is>
       </c>
-      <c r="E37" s="16" t="inlineStr">
+      <c r="E37" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F37" s="16" t="inlineStr">
+      <c r="F37" s="20" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="G37" s="16" t="inlineStr">
+      <c r="G37" s="20" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="H37" s="16" t="inlineStr">
+      <c r="H37" s="20" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
       </c>
-      <c r="I37" s="17" t="n">
+      <c r="I37" s="21" t="n">
         <v>1</v>
       </c>
       <c r="J37" s="8" t="inlineStr">
@@ -2138,12 +2144,12 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="16" t="inlineStr">
+      <c r="A38" s="20" t="inlineStr">
         <is>
           <t>6.2</t>
         </is>
       </c>
-      <c r="B38" s="16" t="inlineStr">
+      <c r="B38" s="20" t="inlineStr">
         <is>
           <t>실제 AI 연결</t>
         </is>
@@ -2158,31 +2164,31 @@
           <t>준비도 기준·항목 가중치·프롬프트를 시나리오로 측정</t>
         </is>
       </c>
-      <c r="E38" s="16" t="inlineStr">
+      <c r="E38" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F38" s="16" t="n"/>
-      <c r="G38" s="16" t="n"/>
-      <c r="H38" s="16" t="inlineStr">
+      <c r="F38" s="20" t="n"/>
+      <c r="G38" s="20" t="n"/>
+      <c r="H38" s="20" t="inlineStr">
         <is>
           <t>예정</t>
         </is>
       </c>
-      <c r="I38" s="17" t="n">
+      <c r="I38" s="21" t="n">
         <v>0</v>
       </c>
       <c r="J38" s="8" t="n"/>
       <c r="K38" s="8" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="16" t="inlineStr">
+      <c r="A39" s="20" t="inlineStr">
         <is>
           <t>6.3</t>
         </is>
       </c>
-      <c r="B39" s="16" t="inlineStr">
+      <c r="B39" s="20" t="inlineStr">
         <is>
           <t>실제 AI 연결</t>
         </is>
@@ -2197,129 +2203,176 @@
           <t>지금의 자리표시·샘플 자리에 실제 기능 연결</t>
         </is>
       </c>
-      <c r="E39" s="16" t="inlineStr">
+      <c r="E39" s="20" t="inlineStr">
         <is>
           <t>개발</t>
         </is>
       </c>
-      <c r="F39" s="16" t="n"/>
-      <c r="G39" s="16" t="n"/>
-      <c r="H39" s="16" t="inlineStr">
+      <c r="F39" s="20" t="n"/>
+      <c r="G39" s="20" t="n"/>
+      <c r="H39" s="20" t="inlineStr">
         <is>
           <t>예정</t>
         </is>
       </c>
-      <c r="I39" s="17" t="n">
+      <c r="I39" s="21" t="n">
         <v>0</v>
       </c>
       <c r="J39" s="8" t="n"/>
       <c r="K39" s="8" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+      <c r="A40" s="20" t="inlineStr">
+        <is>
+          <t>6.4</t>
+        </is>
+      </c>
+      <c r="B40" s="20" t="inlineStr">
+        <is>
+          <t>실제 AI 연결</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>외부 전송 보호(개인정보 가림·비공개·동의)</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="n"/>
+      <c r="E40" s="20" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F40" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="G40" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="H40" s="20" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I40" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J40" s="8" t="inlineStr">
+        <is>
+          <t>PR #24</t>
+        </is>
+      </c>
+      <c r="K40" s="8" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B40" s="4" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>마무리</t>
         </is>
       </c>
-      <c r="C40" s="5" t="inlineStr">
+      <c r="C41" s="5" t="inlineStr">
         <is>
           <t>평가·발표</t>
         </is>
       </c>
-      <c r="D40" s="5" t="n"/>
-      <c r="E40" s="4" t="n"/>
-      <c r="F40" s="4" t="n"/>
-      <c r="G40" s="4" t="n"/>
-      <c r="H40" s="4" t="n"/>
-      <c r="I40" s="6">
-        <f>IFERROR(AVERAGE(I41:I42),0)</f>
-        <v/>
-      </c>
-      <c r="J40" s="5" t="n"/>
-      <c r="K40" s="5" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="16" t="inlineStr">
+      <c r="D41" s="5" t="n"/>
+      <c r="E41" s="4" t="n"/>
+      <c r="F41" s="4" t="n"/>
+      <c r="G41" s="4" t="n"/>
+      <c r="H41" s="4" t="n"/>
+      <c r="I41" s="6">
+        <f>IFERROR(AVERAGE(I42:I43),0)</f>
+        <v/>
+      </c>
+      <c r="J41" s="5" t="n"/>
+      <c r="K41" s="5" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="20" t="inlineStr">
         <is>
           <t>7.1</t>
         </is>
       </c>
-      <c r="B41" s="16" t="inlineStr">
+      <c r="B42" s="20" t="inlineStr">
         <is>
           <t>마무리</t>
         </is>
       </c>
-      <c r="C41" s="8" t="inlineStr">
+      <c r="C42" s="8" t="inlineStr">
         <is>
           <t>사용성 확인·평가 지표 측정</t>
         </is>
       </c>
-      <c r="D41" s="8" t="inlineStr">
+      <c r="D42" s="8" t="inlineStr">
         <is>
           <t>필수정보 충족률, 질문 효율, 가정 표시율 등(기획서 14장)</t>
         </is>
       </c>
-      <c r="E41" s="16" t="inlineStr">
+      <c r="E42" s="20" t="inlineStr">
         <is>
           <t>공동</t>
         </is>
       </c>
-      <c r="F41" s="16" t="n"/>
-      <c r="G41" s="16" t="n"/>
-      <c r="H41" s="16" t="inlineStr">
+      <c r="F42" s="20" t="n"/>
+      <c r="G42" s="20" t="n"/>
+      <c r="H42" s="20" t="inlineStr">
         <is>
           <t>예정</t>
         </is>
       </c>
-      <c r="I41" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J41" s="8" t="n"/>
-      <c r="K41" s="8" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="16" t="inlineStr">
-        <is>
-          <t>7.2</t>
-        </is>
-      </c>
-      <c r="B42" s="16" t="inlineStr">
-        <is>
-          <t>마무리</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>최종 발표 자료</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="n"/>
-      <c r="E42" s="16" t="inlineStr">
-        <is>
-          <t>공동</t>
-        </is>
-      </c>
-      <c r="F42" s="16" t="n"/>
-      <c r="G42" s="16" t="n"/>
-      <c r="H42" s="16" t="inlineStr">
-        <is>
-          <t>예정</t>
-        </is>
-      </c>
-      <c r="I42" s="17" t="n">
+      <c r="I42" s="21" t="n">
         <v>0</v>
       </c>
       <c r="J42" s="8" t="n"/>
       <c r="K42" s="8" t="n"/>
     </row>
+    <row r="43">
+      <c r="A43" s="20" t="inlineStr">
+        <is>
+          <t>7.2</t>
+        </is>
+      </c>
+      <c r="B43" s="20" t="inlineStr">
+        <is>
+          <t>마무리</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>최종 발표 자료</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="n"/>
+      <c r="E43" s="20" t="inlineStr">
+        <is>
+          <t>공동</t>
+        </is>
+      </c>
+      <c r="F43" s="20" t="n"/>
+      <c r="G43" s="20" t="n"/>
+      <c r="H43" s="20" t="inlineStr">
+        <is>
+          <t>예정</t>
+        </is>
+      </c>
+      <c r="I43" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" s="8" t="n"/>
+      <c r="K43" s="8" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:K42"/>
-  <conditionalFormatting sqref="H5:H42">
+  <autoFilter ref="A4:K43"/>
+  <conditionalFormatting sqref="H5:H43">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"완료"</formula>
     </cfRule>
@@ -2330,7 +2383,7 @@
       <formula>"보류"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I42">
+  <conditionalFormatting sqref="I5:I43">
     <cfRule type="dataBar" priority="4">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -2340,10 +2393,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="H5:H42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"완료,진행 중,예정,보류"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E5:E43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"개발,디자인,공동"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2375,7 +2428,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -2415,23 +2467,23 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A4,WBS!$H$5:$H$42,"&lt;&gt;")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A4,WBS!$H$5:$H$43,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C4" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A4,WBS!$H$5:$H$42,"완료")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A4,WBS!$H$5:$H$43,"완료")</f>
         <v/>
       </c>
       <c r="D4" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A4,WBS!$H$5:$H$42,"진행 중")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A4,WBS!$H$5:$H$43,"진행 중")</f>
         <v/>
       </c>
       <c r="E4" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A4,WBS!$H$5:$H$42,"예정")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A4,WBS!$H$5:$H$43,"예정")</f>
         <v/>
       </c>
       <c r="F4" s="12">
-        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$42,WBS!$B$5:$B$42,A4,WBS!$H$5:$H$42,"&lt;&gt;"),0)</f>
+        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$43,WBS!$B$5:$B$43,A4,WBS!$H$5:$H$43,"&lt;&gt;"),0)</f>
         <v/>
       </c>
     </row>
@@ -2442,23 +2494,23 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A5,WBS!$H$5:$H$42,"&lt;&gt;")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A5,WBS!$H$5:$H$43,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C5" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A5,WBS!$H$5:$H$42,"완료")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A5,WBS!$H$5:$H$43,"완료")</f>
         <v/>
       </c>
       <c r="D5" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A5,WBS!$H$5:$H$42,"진행 중")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A5,WBS!$H$5:$H$43,"진행 중")</f>
         <v/>
       </c>
       <c r="E5" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A5,WBS!$H$5:$H$42,"예정")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A5,WBS!$H$5:$H$43,"예정")</f>
         <v/>
       </c>
       <c r="F5" s="12">
-        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$42,WBS!$B$5:$B$42,A5,WBS!$H$5:$H$42,"&lt;&gt;"),0)</f>
+        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$43,WBS!$B$5:$B$43,A5,WBS!$H$5:$H$43,"&lt;&gt;"),0)</f>
         <v/>
       </c>
     </row>
@@ -2469,23 +2521,23 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A6,WBS!$H$5:$H$42,"&lt;&gt;")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A6,WBS!$H$5:$H$43,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C6" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A6,WBS!$H$5:$H$42,"완료")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A6,WBS!$H$5:$H$43,"완료")</f>
         <v/>
       </c>
       <c r="D6" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A6,WBS!$H$5:$H$42,"진행 중")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A6,WBS!$H$5:$H$43,"진행 중")</f>
         <v/>
       </c>
       <c r="E6" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A6,WBS!$H$5:$H$42,"예정")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A6,WBS!$H$5:$H$43,"예정")</f>
         <v/>
       </c>
       <c r="F6" s="12">
-        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$42,WBS!$B$5:$B$42,A6,WBS!$H$5:$H$42,"&lt;&gt;"),0)</f>
+        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$43,WBS!$B$5:$B$43,A6,WBS!$H$5:$H$43,"&lt;&gt;"),0)</f>
         <v/>
       </c>
     </row>
@@ -2496,23 +2548,23 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A7,WBS!$H$5:$H$42,"&lt;&gt;")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A7,WBS!$H$5:$H$43,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C7" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A7,WBS!$H$5:$H$42,"완료")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A7,WBS!$H$5:$H$43,"완료")</f>
         <v/>
       </c>
       <c r="D7" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A7,WBS!$H$5:$H$42,"진행 중")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A7,WBS!$H$5:$H$43,"진행 중")</f>
         <v/>
       </c>
       <c r="E7" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A7,WBS!$H$5:$H$42,"예정")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A7,WBS!$H$5:$H$43,"예정")</f>
         <v/>
       </c>
       <c r="F7" s="12">
-        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$42,WBS!$B$5:$B$42,A7,WBS!$H$5:$H$42,"&lt;&gt;"),0)</f>
+        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$43,WBS!$B$5:$B$43,A7,WBS!$H$5:$H$43,"&lt;&gt;"),0)</f>
         <v/>
       </c>
     </row>
@@ -2523,23 +2575,23 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A8,WBS!$H$5:$H$42,"&lt;&gt;")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A8,WBS!$H$5:$H$43,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C8" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A8,WBS!$H$5:$H$42,"완료")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A8,WBS!$H$5:$H$43,"완료")</f>
         <v/>
       </c>
       <c r="D8" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A8,WBS!$H$5:$H$42,"진행 중")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A8,WBS!$H$5:$H$43,"진행 중")</f>
         <v/>
       </c>
       <c r="E8" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A8,WBS!$H$5:$H$42,"예정")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A8,WBS!$H$5:$H$43,"예정")</f>
         <v/>
       </c>
       <c r="F8" s="12">
-        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$42,WBS!$B$5:$B$42,A8,WBS!$H$5:$H$42,"&lt;&gt;"),0)</f>
+        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$43,WBS!$B$5:$B$43,A8,WBS!$H$5:$H$43,"&lt;&gt;"),0)</f>
         <v/>
       </c>
     </row>
@@ -2550,23 +2602,23 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A9,WBS!$H$5:$H$42,"&lt;&gt;")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A9,WBS!$H$5:$H$43,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C9" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A9,WBS!$H$5:$H$42,"완료")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A9,WBS!$H$5:$H$43,"완료")</f>
         <v/>
       </c>
       <c r="D9" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A9,WBS!$H$5:$H$42,"진행 중")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A9,WBS!$H$5:$H$43,"진행 중")</f>
         <v/>
       </c>
       <c r="E9" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A9,WBS!$H$5:$H$42,"예정")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A9,WBS!$H$5:$H$43,"예정")</f>
         <v/>
       </c>
       <c r="F9" s="12">
-        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$42,WBS!$B$5:$B$42,A9,WBS!$H$5:$H$42,"&lt;&gt;"),0)</f>
+        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$43,WBS!$B$5:$B$43,A9,WBS!$H$5:$H$43,"&lt;&gt;"),0)</f>
         <v/>
       </c>
     </row>
@@ -2577,23 +2629,23 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A10,WBS!$H$5:$H$42,"&lt;&gt;")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A10,WBS!$H$5:$H$43,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C10" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A10,WBS!$H$5:$H$42,"완료")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A10,WBS!$H$5:$H$43,"완료")</f>
         <v/>
       </c>
       <c r="D10" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A10,WBS!$H$5:$H$42,"진행 중")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A10,WBS!$H$5:$H$43,"진행 중")</f>
         <v/>
       </c>
       <c r="E10" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$42,A10,WBS!$H$5:$H$42,"예정")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$43,A10,WBS!$H$5:$H$43,"예정")</f>
         <v/>
       </c>
       <c r="F10" s="12">
-        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$42,WBS!$B$5:$B$42,A10,WBS!$H$5:$H$42,"&lt;&gt;"),0)</f>
+        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$43,WBS!$B$5:$B$43,A10,WBS!$H$5:$H$43,"&lt;&gt;"),0)</f>
         <v/>
       </c>
     </row>
@@ -2620,11 +2672,10 @@
         <v/>
       </c>
       <c r="F11" s="14">
-        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$42,WBS!$H$5:$H$42,"&lt;&gt;"),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12"/>
+        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$43,WBS!$H$5:$H$43,"&lt;&gt;"),0)</f>
+        <v/>
+      </c>
+    </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
데이터 보존: Neon 무료 Postgres(STORE=postgres) (#33)
* 데이터 보존(Neon Postgres) 설계와 구현 계획

* Postgres 세션·결과 이미지 저장소와 계약 테스트

* 저장소 고르기를 build_storage 한 곳으로, STORE=postgres 설정

* Postgres 풀: 죽은 연결 감지, 열기 제한 시간, 파일 id 이름 공개

* Postgres 풀은 서버가 시작할 때 열고 끝날 때 닫는다

* Postgres 연결 끊김 테스트를 풀의 연결 하나로 한정, 풀 열기 실패 시 닫기

* 저장소 닫기를 두 경로 모두에, 열기 판단은 storage.py로

* Postgres 풀은 만들 때 연결하지 않고 서버 시작 때 연다

* 평가 통계도 저장소를 연 뒤 읽는다

* 배포: Neon Postgres로 데이터 보존, 문서·WBS

* Postgres 리뷰 반영: NUL 문자, 테스트 DB 보호, 주소 형식 검사

* 쓰지 않는 import 정리, HANDOFF 테스트 수
</commit_message>
<xml_diff>
--- a/docs/WBS.xlsx
+++ b/docs/WBS.xlsx
@@ -11,7 +11,7 @@
     <sheet name="요약" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WBS'!$A$4:$K$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WBS'!$A$4:$K$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -98,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -129,6 +129,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -589,7 +595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K52"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -705,12 +711,12 @@
       <c r="K5" s="5" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="38" t="inlineStr">
+      <c r="A6" s="40" t="inlineStr">
         <is>
           <t>1.1</t>
         </is>
       </c>
-      <c r="B6" s="38" t="inlineStr">
+      <c r="B6" s="40" t="inlineStr">
         <is>
           <t>기획·설계</t>
         </is>
@@ -725,23 +731,23 @@
           <t>과제 4개(사업계획·상품기획·브랜딩·마케팅), 적응형 질문, 사실·가정 분리 원칙</t>
         </is>
       </c>
-      <c r="E6" s="38" t="inlineStr">
+      <c r="E6" s="40" t="inlineStr">
         <is>
           <t>공동</t>
         </is>
       </c>
-      <c r="F6" s="38" t="n"/>
-      <c r="G6" s="38" t="inlineStr">
+      <c r="F6" s="40" t="n"/>
+      <c r="G6" s="40" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="H6" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I6" s="39" t="n">
+      <c r="H6" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I6" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J6" s="8" t="inlineStr">
@@ -752,12 +758,12 @@
       <c r="K6" s="8" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="38" t="inlineStr">
+      <c r="A7" s="40" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="B7" s="38" t="inlineStr">
+      <c r="B7" s="40" t="inlineStr">
         <is>
           <t>기획·설계</t>
         </is>
@@ -772,27 +778,27 @@
           <t>FastAPI 하네스 구조, API 계약, 테스트 전략</t>
         </is>
       </c>
-      <c r="E7" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F7" s="38" t="inlineStr">
+      <c r="E7" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F7" s="40" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G7" s="38" t="inlineStr">
+      <c r="G7" s="40" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="H7" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I7" s="39" t="n">
+      <c r="H7" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I7" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J7" s="8" t="inlineStr">
@@ -803,12 +809,12 @@
       <c r="K7" s="8" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="38" t="inlineStr">
+      <c r="A8" s="40" t="inlineStr">
         <is>
           <t>1.3</t>
         </is>
       </c>
-      <c r="B8" s="38" t="inlineStr">
+      <c r="B8" s="40" t="inlineStr">
         <is>
           <t>기획·설계</t>
         </is>
@@ -823,27 +829,27 @@
           <t>V2 화면 흐름, 묶음 0~4로 작업 나누기</t>
         </is>
       </c>
-      <c r="E8" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F8" s="38" t="inlineStr">
+      <c r="E8" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F8" s="40" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G8" s="38" t="inlineStr">
+      <c r="G8" s="40" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H8" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I8" s="39" t="n">
+      <c r="H8" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I8" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J8" s="8" t="inlineStr">
@@ -854,12 +860,12 @@
       <c r="K8" s="8" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="38" t="inlineStr">
+      <c r="A9" s="40" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
       </c>
-      <c r="B9" s="38" t="inlineStr">
+      <c r="B9" s="40" t="inlineStr">
         <is>
           <t>기획·설계</t>
         </is>
@@ -874,27 +880,27 @@
           <t>지금 상태·다음 할 일·작업 방식·환경 팁, PR마다 갱신</t>
         </is>
       </c>
-      <c r="E9" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F9" s="38" t="inlineStr">
+      <c r="E9" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F9" s="40" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="G9" s="38" t="inlineStr">
+      <c r="G9" s="40" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="H9" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I9" s="39" t="n">
+      <c r="H9" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I9" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J9" s="8" t="inlineStr">
@@ -905,12 +911,12 @@
       <c r="K9" s="8" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="38" t="inlineStr">
+      <c r="A10" s="40" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="B10" s="38" t="inlineStr">
+      <c r="B10" s="40" t="inlineStr">
         <is>
           <t>기획·설계</t>
         </is>
@@ -925,27 +931,27 @@
           <t>바로 보기 주소, 된 것, 남은 일·맡을 사람·상의할 점</t>
         </is>
       </c>
-      <c r="E10" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F10" s="38" t="inlineStr">
+      <c r="E10" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F10" s="40" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="G10" s="38" t="inlineStr">
+      <c r="G10" s="40" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="H10" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I10" s="39" t="n">
+      <c r="H10" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I10" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J10" s="8" t="inlineStr">
@@ -984,12 +990,12 @@
       <c r="K11" s="5" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="38" t="inlineStr">
+      <c r="A12" s="40" t="inlineStr">
         <is>
           <t>2.1</t>
         </is>
       </c>
-      <c r="B12" s="38" t="inlineStr">
+      <c r="B12" s="40" t="inlineStr">
         <is>
           <t>백엔드 기반</t>
         </is>
@@ -1004,27 +1010,27 @@
           <t>사실·가정·미정 구분, 정보 출처 표시</t>
         </is>
       </c>
-      <c r="E12" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F12" s="38" t="inlineStr">
+      <c r="E12" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F12" s="40" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G12" s="38" t="inlineStr">
+      <c r="G12" s="40" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H12" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I12" s="39" t="n">
+      <c r="H12" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I12" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J12" s="8" t="inlineStr">
@@ -1035,12 +1041,12 @@
       <c r="K12" s="8" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="38" t="inlineStr">
+      <c r="A13" s="40" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="B13" s="38" t="inlineStr">
+      <c r="B13" s="40" t="inlineStr">
         <is>
           <t>백엔드 기반</t>
         </is>
@@ -1055,27 +1061,27 @@
           <t>비용 없이 개발·테스트하는 가짜 모델</t>
         </is>
       </c>
-      <c r="E13" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F13" s="38" t="inlineStr">
+      <c r="E13" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F13" s="40" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="G13" s="38" t="inlineStr">
+      <c r="G13" s="40" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H13" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I13" s="39" t="n">
+      <c r="H13" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I13" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J13" s="8" t="inlineStr">
@@ -1086,12 +1092,12 @@
       <c r="K13" s="8" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="38" t="inlineStr">
+      <c r="A14" s="40" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="B14" s="38" t="inlineStr">
+      <c r="B14" s="40" t="inlineStr">
         <is>
           <t>백엔드 기반</t>
         </is>
@@ -1106,27 +1112,27 @@
           <t>과제별 질문 정책(policy.yaml), 단계별 프롬프트</t>
         </is>
       </c>
-      <c r="E14" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F14" s="38" t="inlineStr">
+      <c r="E14" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F14" s="40" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G14" s="38" t="inlineStr">
+      <c r="G14" s="40" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H14" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I14" s="39" t="n">
+      <c r="H14" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I14" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J14" s="8" t="inlineStr">
@@ -1137,12 +1143,12 @@
       <c r="K14" s="8" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="38" t="inlineStr">
+      <c r="A15" s="40" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="B15" s="38" t="inlineStr">
+      <c r="B15" s="40" t="inlineStr">
         <is>
           <t>백엔드 기반</t>
         </is>
@@ -1157,27 +1163,27 @@
           <t>모드별 질문 상한, '다른 예시 보기' 단계</t>
         </is>
       </c>
-      <c r="E15" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F15" s="38" t="inlineStr">
+      <c r="E15" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F15" s="40" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G15" s="38" t="inlineStr">
+      <c r="G15" s="40" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H15" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I15" s="39" t="n">
+      <c r="H15" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I15" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J15" s="8" t="inlineStr">
@@ -1188,12 +1194,12 @@
       <c r="K15" s="8" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="38" t="inlineStr">
+      <c r="A16" s="40" t="inlineStr">
         <is>
           <t>2.5</t>
         </is>
       </c>
-      <c r="B16" s="38" t="inlineStr">
+      <c r="B16" s="40" t="inlineStr">
         <is>
           <t>백엔드 기반</t>
         </is>
@@ -1204,27 +1210,27 @@
         </is>
       </c>
       <c r="D16" s="8" t="n"/>
-      <c r="E16" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F16" s="38" t="inlineStr">
+      <c r="E16" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F16" s="40" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G16" s="38" t="inlineStr">
+      <c r="G16" s="40" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H16" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I16" s="39" t="n">
+      <c r="H16" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I16" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J16" s="8" t="inlineStr">
@@ -1235,12 +1241,12 @@
       <c r="K16" s="8" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="38" t="inlineStr">
+      <c r="A17" s="40" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="B17" s="38" t="inlineStr">
+      <c r="B17" s="40" t="inlineStr">
         <is>
           <t>백엔드 기반</t>
         </is>
@@ -1255,27 +1261,27 @@
           <t>과제별 정책·프롬프트·검증 규칙</t>
         </is>
       </c>
-      <c r="E17" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F17" s="38" t="inlineStr">
+      <c r="E17" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F17" s="40" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G17" s="38" t="inlineStr">
+      <c r="G17" s="40" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H17" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I17" s="39" t="n">
+      <c r="H17" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I17" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J17" s="8" t="inlineStr">
@@ -1286,12 +1292,12 @@
       <c r="K17" s="8" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="38" t="inlineStr">
+      <c r="A18" s="40" t="inlineStr">
         <is>
           <t>2.7</t>
         </is>
       </c>
-      <c r="B18" s="38" t="inlineStr">
+      <c r="B18" s="40" t="inlineStr">
         <is>
           <t>백엔드 기반</t>
         </is>
@@ -1306,27 +1312,27 @@
           <t>한국어 오류 문구, API 문서</t>
         </is>
       </c>
-      <c r="E18" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F18" s="38" t="inlineStr">
+      <c r="E18" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F18" s="40" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G18" s="38" t="inlineStr">
+      <c r="G18" s="40" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H18" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I18" s="39" t="n">
+      <c r="H18" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I18" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J18" s="8" t="inlineStr">
@@ -1337,12 +1343,12 @@
       <c r="K18" s="8" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="38" t="inlineStr">
+      <c r="A19" s="40" t="inlineStr">
         <is>
           <t>2.8</t>
         </is>
       </c>
-      <c r="B19" s="38" t="inlineStr">
+      <c r="B19" s="40" t="inlineStr">
         <is>
           <t>백엔드 기반</t>
         </is>
@@ -1357,27 +1363,27 @@
           <t>API에 맞춘 최소 화면, 개발 안내(CLAUDE.md)</t>
         </is>
       </c>
-      <c r="E19" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F19" s="38" t="inlineStr">
+      <c r="E19" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F19" s="40" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G19" s="38" t="inlineStr">
+      <c r="G19" s="40" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H19" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I19" s="39" t="n">
+      <c r="H19" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I19" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J19" s="8" t="inlineStr">
@@ -1416,12 +1422,12 @@
       <c r="K20" s="5" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="38" t="inlineStr">
+      <c r="A21" s="40" t="inlineStr">
         <is>
           <t>3.1</t>
         </is>
       </c>
-      <c r="B21" s="38" t="inlineStr">
+      <c r="B21" s="40" t="inlineStr">
         <is>
           <t>디자인</t>
         </is>
@@ -1436,23 +1442,23 @@
           <t>전체 화면 흐름 HTML 프로토타입</t>
         </is>
       </c>
-      <c r="E21" s="38" t="inlineStr">
+      <c r="E21" s="40" t="inlineStr">
         <is>
           <t>디자인</t>
         </is>
       </c>
-      <c r="F21" s="38" t="n"/>
-      <c r="G21" s="38" t="inlineStr">
+      <c r="F21" s="40" t="n"/>
+      <c r="G21" s="40" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H21" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I21" s="39" t="n">
+      <c r="H21" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I21" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J21" s="8" t="inlineStr">
@@ -1463,12 +1469,12 @@
       <c r="K21" s="8" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="38" t="inlineStr">
+      <c r="A22" s="40" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="B22" s="38" t="inlineStr">
+      <c r="B22" s="40" t="inlineStr">
         <is>
           <t>디자인</t>
         </is>
@@ -1483,27 +1489,27 @@
           <t>모든 질문에 '다른 예시 보기', 모드 설명, 이미지 블록, 생성 중·실패·최신 아님 상태</t>
         </is>
       </c>
-      <c r="E22" s="38" t="inlineStr">
+      <c r="E22" s="40" t="inlineStr">
         <is>
           <t>디자인</t>
         </is>
       </c>
-      <c r="F22" s="38" t="inlineStr">
+      <c r="F22" s="40" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="G22" s="38" t="inlineStr">
+      <c r="G22" s="40" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="H22" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I22" s="39" t="n">
+      <c r="H22" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I22" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J22" s="8" t="inlineStr">
@@ -1514,12 +1520,12 @@
       <c r="K22" s="8" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="38" t="inlineStr">
+      <c r="A23" s="40" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
       </c>
-      <c r="B23" s="38" t="inlineStr">
+      <c r="B23" s="40" t="inlineStr">
         <is>
           <t>디자인</t>
         </is>
@@ -1534,31 +1540,31 @@
           <t>반응형 자동 배치 확인</t>
         </is>
       </c>
-      <c r="E23" s="38" t="inlineStr">
+      <c r="E23" s="40" t="inlineStr">
         <is>
           <t>디자인</t>
         </is>
       </c>
-      <c r="F23" s="38" t="n"/>
-      <c r="G23" s="38" t="n"/>
-      <c r="H23" s="38" t="inlineStr">
+      <c r="F23" s="40" t="n"/>
+      <c r="G23" s="40" t="n"/>
+      <c r="H23" s="40" t="inlineStr">
         <is>
           <t>예정</t>
         </is>
       </c>
-      <c r="I23" s="39" t="n">
+      <c r="I23" s="41" t="n">
         <v>0</v>
       </c>
       <c r="J23" s="8" t="n"/>
       <c r="K23" s="8" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="38" t="inlineStr">
+      <c r="A24" s="40" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>
       </c>
-      <c r="B24" s="38" t="inlineStr">
+      <c r="B24" s="40" t="inlineStr">
         <is>
           <t>디자인</t>
         </is>
@@ -1573,19 +1579,19 @@
           <t>/preview 화면을 html.to.design으로 가져와 수정</t>
         </is>
       </c>
-      <c r="E24" s="38" t="inlineStr">
+      <c r="E24" s="40" t="inlineStr">
         <is>
           <t>디자인</t>
         </is>
       </c>
-      <c r="F24" s="38" t="n"/>
-      <c r="G24" s="38" t="n"/>
-      <c r="H24" s="38" t="inlineStr">
+      <c r="F24" s="40" t="n"/>
+      <c r="G24" s="40" t="n"/>
+      <c r="H24" s="40" t="inlineStr">
         <is>
           <t>예정</t>
         </is>
       </c>
-      <c r="I24" s="39" t="n">
+      <c r="I24" s="41" t="n">
         <v>0</v>
       </c>
       <c r="J24" s="8" t="n"/>
@@ -1620,12 +1626,12 @@
       <c r="K25" s="5" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="38" t="inlineStr">
+      <c r="A26" s="40" t="inlineStr">
         <is>
           <t>4.1</t>
         </is>
       </c>
-      <c r="B26" s="38" t="inlineStr">
+      <c r="B26" s="40" t="inlineStr">
         <is>
           <t>화면 개발(V2)</t>
         </is>
@@ -1640,27 +1646,27 @@
           <t>버셀 배포 설정 포함</t>
         </is>
       </c>
-      <c r="E26" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F26" s="38" t="inlineStr">
+      <c r="E26" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F26" s="40" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="G26" s="38" t="inlineStr">
+      <c r="G26" s="40" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="H26" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I26" s="39" t="n">
+      <c r="H26" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I26" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J26" s="8" t="inlineStr">
@@ -1671,12 +1677,12 @@
       <c r="K26" s="8" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="38" t="inlineStr">
+      <c r="A27" s="40" t="inlineStr">
         <is>
           <t>4.2</t>
         </is>
       </c>
-      <c r="B27" s="38" t="inlineStr">
+      <c r="B27" s="40" t="inlineStr">
         <is>
           <t>화면 개발(V2)</t>
         </is>
@@ -1691,27 +1697,27 @@
           <t>답변 종류, 흐름 패널, 익명 사용자</t>
         </is>
       </c>
-      <c r="E27" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F27" s="38" t="inlineStr">
+      <c r="E27" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F27" s="40" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="G27" s="38" t="inlineStr">
+      <c r="G27" s="40" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="H27" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I27" s="39" t="n">
+      <c r="H27" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I27" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J27" s="8" t="inlineStr">
@@ -1722,12 +1728,12 @@
       <c r="K27" s="8" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="38" t="inlineStr">
+      <c r="A28" s="40" t="inlineStr">
         <is>
           <t>4.3</t>
         </is>
       </c>
-      <c r="B28" s="38" t="inlineStr">
+      <c r="B28" s="40" t="inlineStr">
         <is>
           <t>화면 개발(V2)</t>
         </is>
@@ -1742,27 +1748,27 @@
           <t>서버 저장(SQLite), 문서 내려받기</t>
         </is>
       </c>
-      <c r="E28" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F28" s="38" t="inlineStr">
+      <c r="E28" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F28" s="40" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="G28" s="38" t="inlineStr">
+      <c r="G28" s="40" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="H28" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I28" s="39" t="n">
+      <c r="H28" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I28" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J28" s="8" t="inlineStr">
@@ -1773,12 +1779,12 @@
       <c r="K28" s="8" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="38" t="inlineStr">
+      <c r="A29" s="40" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
       </c>
-      <c r="B29" s="38" t="inlineStr">
+      <c r="B29" s="40" t="inlineStr">
         <is>
           <t>화면 개발(V2)</t>
         </is>
@@ -1793,27 +1799,27 @@
           <t>결과를 섹션·블록으로</t>
         </is>
       </c>
-      <c r="E29" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F29" s="38" t="inlineStr">
+      <c r="E29" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F29" s="40" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="G29" s="38" t="inlineStr">
+      <c r="G29" s="40" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="H29" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I29" s="39" t="n">
+      <c r="H29" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I29" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J29" s="8" t="inlineStr">
@@ -1824,12 +1830,12 @@
       <c r="K29" s="8" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="38" t="inlineStr">
+      <c r="A30" s="40" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="B30" s="38" t="inlineStr">
+      <c r="B30" s="40" t="inlineStr">
         <is>
           <t>화면 개발(V2)</t>
         </is>
@@ -1844,27 +1850,27 @@
           <t>샘플 근거 자료, 자리표시 이미지</t>
         </is>
       </c>
-      <c r="E30" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F30" s="38" t="inlineStr">
+      <c r="E30" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F30" s="40" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="G30" s="38" t="inlineStr">
+      <c r="G30" s="40" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="H30" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I30" s="39" t="n">
+      <c r="H30" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I30" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J30" s="8" t="inlineStr">
@@ -1875,12 +1881,12 @@
       <c r="K30" s="8" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="38" t="inlineStr">
+      <c r="A31" s="40" t="inlineStr">
         <is>
           <t>4.6</t>
         </is>
       </c>
-      <c r="B31" s="38" t="inlineStr">
+      <c r="B31" s="40" t="inlineStr">
         <is>
           <t>화면 개발(V2)</t>
         </is>
@@ -1895,27 +1901,27 @@
           <t>생성 중·생성 실패 화면, 최신 아님 배너, 이미지 상자, 모드 설명</t>
         </is>
       </c>
-      <c r="E31" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F31" s="38" t="inlineStr">
+      <c r="E31" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F31" s="40" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="G31" s="38" t="inlineStr">
+      <c r="G31" s="40" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="H31" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I31" s="39" t="n">
+      <c r="H31" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I31" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J31" s="8" t="inlineStr">
@@ -1926,12 +1932,12 @@
       <c r="K31" s="8" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="38" t="inlineStr">
+      <c r="A32" s="40" t="inlineStr">
         <is>
           <t>4.7</t>
         </is>
       </c>
-      <c r="B32" s="38" t="inlineStr">
+      <c r="B32" s="40" t="inlineStr">
         <is>
           <t>화면 개발(V2)</t>
         </is>
@@ -1946,27 +1952,27 @@
           <t>이전 결과를 다음 과제의 기준으로 가져오기</t>
         </is>
       </c>
-      <c r="E32" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F32" s="38" t="inlineStr">
+      <c r="E32" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F32" s="40" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="G32" s="38" t="inlineStr">
+      <c r="G32" s="40" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="H32" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I32" s="39" t="n">
+      <c r="H32" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I32" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J32" s="8" t="inlineStr">
@@ -1977,12 +1983,12 @@
       <c r="K32" s="8" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="38" t="inlineStr">
+      <c r="A33" s="40" t="inlineStr">
         <is>
           <t>4.8</t>
         </is>
       </c>
-      <c r="B33" s="38" t="inlineStr">
+      <c r="B33" s="40" t="inlineStr">
         <is>
           <t>화면 개발(V2)</t>
         </is>
@@ -1993,27 +1999,27 @@
         </is>
       </c>
       <c r="D33" s="8" t="n"/>
-      <c r="E33" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F33" s="38" t="inlineStr">
+      <c r="E33" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F33" s="40" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="G33" s="38" t="inlineStr">
+      <c r="G33" s="40" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="H33" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I33" s="39" t="n">
+      <c r="H33" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I33" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J33" s="8" t="inlineStr">
@@ -2028,12 +2034,12 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="38" t="inlineStr">
+      <c r="A34" s="40" t="inlineStr">
         <is>
           <t>4.9</t>
         </is>
       </c>
-      <c r="B34" s="38" t="inlineStr">
+      <c r="B34" s="40" t="inlineStr">
         <is>
           <t>화면 개발(V2)</t>
         </is>
@@ -2044,23 +2050,23 @@
         </is>
       </c>
       <c r="D34" s="8" t="n"/>
-      <c r="E34" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F34" s="38" t="n"/>
-      <c r="G34" s="38" t="inlineStr">
+      <c r="E34" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F34" s="40" t="n"/>
+      <c r="G34" s="40" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="H34" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I34" s="39" t="n">
+      <c r="H34" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I34" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J34" s="8" t="inlineStr">
@@ -2071,12 +2077,12 @@
       <c r="K34" s="8" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="38" t="inlineStr">
+      <c r="A35" s="40" t="inlineStr">
         <is>
           <t>4.10</t>
         </is>
       </c>
-      <c r="B35" s="38" t="inlineStr">
+      <c r="B35" s="40" t="inlineStr">
         <is>
           <t>화면 개발(V2)</t>
         </is>
@@ -2087,31 +2093,31 @@
         </is>
       </c>
       <c r="D35" s="8" t="n"/>
-      <c r="E35" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F35" s="38" t="n"/>
-      <c r="G35" s="38" t="n"/>
-      <c r="H35" s="38" t="inlineStr">
+      <c r="E35" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F35" s="40" t="n"/>
+      <c r="G35" s="40" t="n"/>
+      <c r="H35" s="40" t="inlineStr">
         <is>
           <t>예정</t>
         </is>
       </c>
-      <c r="I35" s="39" t="n">
+      <c r="I35" s="41" t="n">
         <v>0</v>
       </c>
       <c r="J35" s="8" t="n"/>
       <c r="K35" s="8" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="38" t="inlineStr">
+      <c r="A36" s="40" t="inlineStr">
         <is>
           <t>4.11</t>
         </is>
       </c>
-      <c r="B36" s="38" t="inlineStr">
+      <c r="B36" s="40" t="inlineStr">
         <is>
           <t>화면 개발(V2)</t>
         </is>
@@ -2122,19 +2128,19 @@
         </is>
       </c>
       <c r="D36" s="8" t="n"/>
-      <c r="E36" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F36" s="38" t="n"/>
-      <c r="G36" s="38" t="n"/>
-      <c r="H36" s="38" t="inlineStr">
+      <c r="E36" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F36" s="40" t="n"/>
+      <c r="G36" s="40" t="n"/>
+      <c r="H36" s="40" t="inlineStr">
         <is>
           <t>예정</t>
         </is>
       </c>
-      <c r="I36" s="39" t="n">
+      <c r="I36" s="41" t="n">
         <v>0</v>
       </c>
       <c r="J36" s="8" t="n"/>
@@ -2162,19 +2168,19 @@
       <c r="G37" s="4" t="n"/>
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="6">
-        <f>IFERROR(AVERAGE(I38:I39),0)</f>
+        <f>IFERROR(AVERAGE(I38:I40),0)</f>
         <v/>
       </c>
       <c r="J37" s="5" t="n"/>
       <c r="K37" s="5" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="38" t="inlineStr">
+      <c r="A38" s="40" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
       </c>
-      <c r="B38" s="38" t="inlineStr">
+      <c r="B38" s="40" t="inlineStr">
         <is>
           <t>배포</t>
         </is>
@@ -2189,27 +2195,27 @@
           <t>main은 정식 주소, PR마다 미리보기 주소</t>
         </is>
       </c>
-      <c r="E38" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F38" s="38" t="inlineStr">
+      <c r="E38" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F38" s="40" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="G38" s="38" t="inlineStr">
+      <c r="G38" s="40" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="H38" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I38" s="39" t="n">
+      <c r="H38" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I38" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J38" s="8" t="inlineStr">
@@ -2224,12 +2230,12 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="38" t="inlineStr">
+      <c r="A39" s="40" t="inlineStr">
         <is>
           <t>5.2</t>
         </is>
       </c>
-      <c r="B39" s="38" t="inlineStr">
+      <c r="B39" s="40" t="inlineStr">
         <is>
           <t>배포</t>
         </is>
@@ -2244,27 +2250,27 @@
           <t>저장 디스크 방식 정하기, 프론트와 연결</t>
         </is>
       </c>
-      <c r="E39" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F39" s="38" t="inlineStr">
+      <c r="E39" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F39" s="40" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="G39" s="38" t="inlineStr">
+      <c r="G39" s="40" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="H39" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I39" s="39" t="n">
+      <c r="H39" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I39" s="41" t="n">
         <v>1</v>
       </c>
       <c r="J39" s="8" t="inlineStr">
@@ -2279,585 +2285,632 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+      <c r="A40" s="40" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="B40" s="40" t="inlineStr">
+        <is>
+          <t>배포</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>데이터 보존(Neon Postgres)</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="n"/>
+      <c r="E40" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F40" s="40" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="G40" s="40" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H40" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I40" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="J40" s="8" t="inlineStr">
+        <is>
+          <t>PR #33</t>
+        </is>
+      </c>
+      <c r="K40" s="8" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B40" s="4" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>실제 AI 연결</t>
         </is>
       </c>
-      <c r="C40" s="5" t="inlineStr">
+      <c r="C41" s="5" t="inlineStr">
         <is>
           <t>실제 AI 연결·튜닝</t>
         </is>
       </c>
-      <c r="D40" s="5" t="n"/>
-      <c r="E40" s="4" t="n"/>
-      <c r="F40" s="4" t="n"/>
-      <c r="G40" s="4" t="n"/>
-      <c r="H40" s="4" t="n"/>
-      <c r="I40" s="6">
-        <f>IFERROR(AVERAGE(I41:I49),0)</f>
-        <v/>
-      </c>
-      <c r="J40" s="5" t="n"/>
-      <c r="K40" s="5" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="38" t="inlineStr">
+      <c r="D41" s="5" t="n"/>
+      <c r="E41" s="4" t="n"/>
+      <c r="F41" s="4" t="n"/>
+      <c r="G41" s="4" t="n"/>
+      <c r="H41" s="4" t="n"/>
+      <c r="I41" s="6">
+        <f>IFERROR(AVERAGE(I42:I50),0)</f>
+        <v/>
+      </c>
+      <c r="J41" s="5" t="n"/>
+      <c r="K41" s="5" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="40" t="inlineStr">
         <is>
           <t>6.1</t>
         </is>
       </c>
-      <c r="B41" s="38" t="inlineStr">
+      <c r="B42" s="40" t="inlineStr">
         <is>
           <t>실제 AI 연결</t>
         </is>
       </c>
-      <c r="C41" s="8" t="inlineStr">
+      <c r="C42" s="8" t="inlineStr">
         <is>
           <t>Claude 모델 연결</t>
         </is>
       </c>
-      <c r="D41" s="8" t="inlineStr">
+      <c r="D42" s="8" t="inlineStr">
         <is>
           <t>가짜 모델(Mock) 대신 실제 모델</t>
         </is>
       </c>
-      <c r="E41" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F41" s="38" t="inlineStr">
+      <c r="E42" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F42" s="40" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="G41" s="38" t="inlineStr">
+      <c r="G42" s="40" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="H41" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I41" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="J41" s="8" t="inlineStr">
+      <c r="H42" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I42" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="J42" s="8" t="inlineStr">
         <is>
           <t>PR #20</t>
         </is>
       </c>
-      <c r="K41" s="8" t="inlineStr">
+      <c r="K42" s="8" t="inlineStr">
         <is>
           <t>어댑터 준비(기본 Mock). 실제 호출·모델·비용은 인수 기업</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="38" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="40" t="inlineStr">
         <is>
           <t>6.2</t>
         </is>
       </c>
-      <c r="B42" s="38" t="inlineStr">
+      <c r="B43" s="40" t="inlineStr">
         <is>
           <t>실제 AI 연결</t>
         </is>
       </c>
-      <c r="C42" s="8" t="inlineStr">
+      <c r="C43" s="8" t="inlineStr">
         <is>
           <t>과제별 질문·결과 품질 튜닝</t>
         </is>
       </c>
-      <c r="D42" s="8" t="inlineStr">
+      <c r="D43" s="8" t="inlineStr">
         <is>
           <t>준비도 기준·항목 가중치·프롬프트를 시나리오로 측정</t>
         </is>
       </c>
-      <c r="E42" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F42" s="38" t="n"/>
-      <c r="G42" s="38" t="n"/>
-      <c r="H42" s="38" t="inlineStr">
+      <c r="E43" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F43" s="40" t="n"/>
+      <c r="G43" s="40" t="n"/>
+      <c r="H43" s="40" t="inlineStr">
         <is>
           <t>예정</t>
         </is>
       </c>
-      <c r="I42" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="J42" s="8" t="n"/>
-      <c r="K42" s="8" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="38" t="inlineStr">
-        <is>
-          <t>6.3</t>
-        </is>
-      </c>
-      <c r="B43" s="38" t="inlineStr">
-        <is>
-          <t>실제 AI 연결</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>이미지 생성·웹 검색 근거 연결</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>지금의 자리표시·샘플 자리에 실제 기능 연결</t>
-        </is>
-      </c>
-      <c r="E43" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F43" s="38" t="n"/>
-      <c r="G43" s="38" t="n"/>
-      <c r="H43" s="38" t="inlineStr">
-        <is>
-          <t>예정</t>
-        </is>
-      </c>
-      <c r="I43" s="39" t="n">
+      <c r="I43" s="41" t="n">
         <v>0</v>
       </c>
       <c r="J43" s="8" t="n"/>
       <c r="K43" s="8" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="38" t="inlineStr">
+      <c r="A44" s="40" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="B44" s="40" t="inlineStr">
+        <is>
+          <t>실제 AI 연결</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>이미지 생성·웹 검색 근거 연결</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>지금의 자리표시·샘플 자리에 실제 기능 연결</t>
+        </is>
+      </c>
+      <c r="E44" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F44" s="40" t="n"/>
+      <c r="G44" s="40" t="n"/>
+      <c r="H44" s="40" t="inlineStr">
+        <is>
+          <t>예정</t>
+        </is>
+      </c>
+      <c r="I44" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" s="8" t="n"/>
+      <c r="K44" s="8" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="40" t="inlineStr">
         <is>
           <t>6.4</t>
         </is>
       </c>
-      <c r="B44" s="38" t="inlineStr">
+      <c r="B45" s="40" t="inlineStr">
         <is>
           <t>실제 AI 연결</t>
         </is>
       </c>
-      <c r="C44" s="8" t="inlineStr">
+      <c r="C45" s="8" t="inlineStr">
         <is>
           <t>외부 전송 보호(개인정보 가림·비공개·동의)</t>
         </is>
       </c>
-      <c r="D44" s="8" t="n"/>
-      <c r="E44" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F44" s="38" t="inlineStr">
+      <c r="D45" s="8" t="n"/>
+      <c r="E45" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F45" s="40" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="G44" s="38" t="inlineStr">
+      <c r="G45" s="40" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="H44" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I44" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="J44" s="8" t="inlineStr">
+      <c r="H45" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I45" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="J45" s="8" t="inlineStr">
         <is>
           <t>PR #24</t>
         </is>
       </c>
-      <c r="K44" s="8" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="38" t="inlineStr">
+      <c r="K45" s="8" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="40" t="inlineStr">
         <is>
           <t>6.5</t>
         </is>
       </c>
-      <c r="B45" s="38" t="inlineStr">
+      <c r="B46" s="40" t="inlineStr">
         <is>
           <t>실제 AI 연결</t>
         </is>
       </c>
-      <c r="C45" s="8" t="inlineStr">
+      <c r="C46" s="8" t="inlineStr">
         <is>
           <t>프롬프트 주입 기본 방어(입력 감싸기·유출 차단)</t>
         </is>
       </c>
-      <c r="D45" s="8" t="n"/>
-      <c r="E45" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F45" s="38" t="inlineStr">
+      <c r="D46" s="8" t="n"/>
+      <c r="E46" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F46" s="40" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="G45" s="38" t="inlineStr">
+      <c r="G46" s="40" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="H45" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I45" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="J45" s="8" t="inlineStr">
+      <c r="H46" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I46" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="J46" s="8" t="inlineStr">
         <is>
           <t>PR #25</t>
         </is>
       </c>
-      <c r="K45" s="8" t="inlineStr">
+      <c r="K46" s="8" t="inlineStr">
         <is>
           <t>PR #25</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="38" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="40" t="inlineStr">
         <is>
           <t>6.6</t>
         </is>
       </c>
-      <c r="B46" s="38" t="inlineStr">
+      <c r="B47" s="40" t="inlineStr">
         <is>
           <t>실제 AI 연결</t>
         </is>
       </c>
-      <c r="C46" s="8" t="inlineStr">
+      <c r="C47" s="8" t="inlineStr">
         <is>
           <t>단계별 모델 라우팅·하네스 로드맵·인수 안내</t>
         </is>
       </c>
-      <c r="D46" s="8" t="n"/>
-      <c r="E46" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F46" s="38" t="inlineStr">
+      <c r="D47" s="8" t="n"/>
+      <c r="E47" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F47" s="40" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="G46" s="38" t="inlineStr">
+      <c r="G47" s="40" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="H46" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I46" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="J46" s="8" t="inlineStr">
+      <c r="H47" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I47" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="J47" s="8" t="inlineStr">
         <is>
           <t>PR #26</t>
         </is>
       </c>
-      <c r="K46" s="8" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="38" t="inlineStr">
+      <c r="K47" s="8" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="40" t="inlineStr">
         <is>
           <t>6.7</t>
         </is>
       </c>
-      <c r="B47" s="38" t="inlineStr">
+      <c r="B48" s="40" t="inlineStr">
         <is>
           <t>실제 AI 연결</t>
         </is>
       </c>
-      <c r="C47" s="8" t="inlineStr">
+      <c r="C48" s="8" t="inlineStr">
         <is>
           <t>AI 동시 호출 상한(붐비면 503)</t>
         </is>
       </c>
-      <c r="D47" s="8" t="inlineStr">
+      <c r="D48" s="8" t="inlineStr">
         <is>
           <t>LLM·이미지 호출 자리 수 제한, 대기 뒤 거절, 세션 되돌림</t>
         </is>
       </c>
-      <c r="E47" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F47" s="38" t="inlineStr">
+      <c r="E48" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F48" s="40" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="G47" s="38" t="inlineStr">
+      <c r="G48" s="40" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="H47" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I47" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="J47" s="8" t="inlineStr">
+      <c r="H48" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I48" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="J48" s="8" t="inlineStr">
         <is>
           <t>PR #27</t>
         </is>
       </c>
-      <c r="K47" s="8" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="38" t="inlineStr">
+      <c r="K48" s="8" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="40" t="inlineStr">
         <is>
           <t>6.8</t>
         </is>
       </c>
-      <c r="B48" s="38" t="inlineStr">
+      <c r="B49" s="40" t="inlineStr">
         <is>
           <t>실제 AI 연결</t>
         </is>
       </c>
-      <c r="C48" s="8" t="inlineStr">
+      <c r="C49" s="8" t="inlineStr">
         <is>
           <t>병렬 생성(기본 꺼짐)·설계 고민 기록</t>
         </is>
       </c>
-      <c r="D48" s="8" t="inlineStr">
+      <c r="D49" s="8" t="inlineStr">
         <is>
           <t>결과 항목 조각 동시 생성·코드 합치기·부분 결과 캐시, README 설계 고민, 로드맵 측정표</t>
         </is>
       </c>
-      <c r="E48" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F48" s="38" t="inlineStr">
+      <c r="E49" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F49" s="40" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="G48" s="38" t="inlineStr">
+      <c r="G49" s="40" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="H48" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I48" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="J48" s="8" t="inlineStr">
+      <c r="H49" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I49" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="J49" s="8" t="inlineStr">
         <is>
           <t>PR #28</t>
         </is>
       </c>
-      <c r="K48" s="8" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="38" t="inlineStr">
+      <c r="K49" s="8" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="40" t="inlineStr">
         <is>
           <t>6.9</t>
         </is>
       </c>
-      <c r="B49" s="38" t="inlineStr">
+      <c r="B50" s="40" t="inlineStr">
         <is>
           <t>실제 AI 연결</t>
         </is>
       </c>
-      <c r="C49" s="8" t="inlineStr">
+      <c r="C50" s="8" t="inlineStr">
         <is>
           <t>측정 준비(응답 시간 기록·측정 도구)</t>
         </is>
       </c>
-      <c r="D49" s="8" t="inlineStr">
+      <c r="D50" s="8" t="inlineStr">
         <is>
           <t>trace duration_ms, 실제 모델용 시나리오 실행, quick-skip 시나리오, scripts/measure.py(기본 Mock, 비용 상한)</t>
         </is>
       </c>
-      <c r="E49" s="38" t="inlineStr">
-        <is>
-          <t>개발</t>
-        </is>
-      </c>
-      <c r="F49" s="38" t="inlineStr">
+      <c r="E50" s="40" t="inlineStr">
+        <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="F50" s="40" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="G49" s="38" t="inlineStr">
+      <c r="G50" s="40" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="H49" s="38" t="inlineStr">
-        <is>
-          <t>완료</t>
-        </is>
-      </c>
-      <c r="I49" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="J49" s="8" t="inlineStr">
+      <c r="H50" s="40" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="I50" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="J50" s="8" t="inlineStr">
         <is>
           <t>PR #29</t>
         </is>
       </c>
-      <c r="K49" s="8" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+      <c r="K50" s="8" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>마무리</t>
         </is>
       </c>
-      <c r="C50" s="5" t="inlineStr">
+      <c r="C51" s="5" t="inlineStr">
         <is>
           <t>평가·발표</t>
         </is>
       </c>
-      <c r="D50" s="5" t="n"/>
-      <c r="E50" s="4" t="n"/>
-      <c r="F50" s="4" t="n"/>
-      <c r="G50" s="4" t="n"/>
-      <c r="H50" s="4" t="n"/>
-      <c r="I50" s="6">
-        <f>IFERROR(AVERAGE(I51:I52),0)</f>
-        <v/>
-      </c>
-      <c r="J50" s="5" t="n"/>
-      <c r="K50" s="5" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="38" t="inlineStr">
+      <c r="D51" s="5" t="n"/>
+      <c r="E51" s="4" t="n"/>
+      <c r="F51" s="4" t="n"/>
+      <c r="G51" s="4" t="n"/>
+      <c r="H51" s="4" t="n"/>
+      <c r="I51" s="6">
+        <f>IFERROR(AVERAGE(I52:I53),0)</f>
+        <v/>
+      </c>
+      <c r="J51" s="5" t="n"/>
+      <c r="K51" s="5" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="40" t="inlineStr">
         <is>
           <t>7.1</t>
         </is>
       </c>
-      <c r="B51" s="38" t="inlineStr">
+      <c r="B52" s="40" t="inlineStr">
         <is>
           <t>마무리</t>
         </is>
       </c>
-      <c r="C51" s="8" t="inlineStr">
+      <c r="C52" s="8" t="inlineStr">
         <is>
           <t>사용성 확인·평가 지표 측정</t>
         </is>
       </c>
-      <c r="D51" s="8" t="inlineStr">
+      <c r="D52" s="8" t="inlineStr">
         <is>
           <t>필수정보 충족률, 질문 효율, 가정 표시율 등(기획서 14장)</t>
         </is>
       </c>
-      <c r="E51" s="38" t="inlineStr">
+      <c r="E52" s="40" t="inlineStr">
         <is>
           <t>공동</t>
         </is>
       </c>
-      <c r="F51" s="38" t="inlineStr">
+      <c r="F52" s="40" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="G51" s="38" t="n"/>
-      <c r="H51" s="38" t="inlineStr">
+      <c r="G52" s="40" t="n"/>
+      <c r="H52" s="40" t="inlineStr">
         <is>
           <t>진행 중</t>
         </is>
       </c>
-      <c r="I51" s="39" t="n">
+      <c r="I52" s="41" t="n">
         <v>0.3</v>
       </c>
-      <c r="J51" s="8" t="inlineStr">
+      <c r="J52" s="8" t="inlineStr">
         <is>
           <t>PR #30 평가 계획·통계 도구</t>
         </is>
       </c>
-      <c r="K51" s="8" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="38" t="inlineStr">
+      <c r="K52" s="8" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="40" t="inlineStr">
         <is>
           <t>7.2</t>
         </is>
       </c>
-      <c r="B52" s="38" t="inlineStr">
+      <c r="B53" s="40" t="inlineStr">
         <is>
           <t>마무리</t>
         </is>
       </c>
-      <c r="C52" s="8" t="inlineStr">
+      <c r="C53" s="8" t="inlineStr">
         <is>
           <t>최종 발표 자료</t>
         </is>
       </c>
-      <c r="D52" s="8" t="n"/>
-      <c r="E52" s="38" t="inlineStr">
+      <c r="D53" s="8" t="n"/>
+      <c r="E53" s="40" t="inlineStr">
         <is>
           <t>공동</t>
         </is>
       </c>
-      <c r="F52" s="38" t="inlineStr">
+      <c r="F53" s="40" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="G52" s="38" t="n"/>
-      <c r="H52" s="38" t="inlineStr">
+      <c r="G53" s="40" t="n"/>
+      <c r="H53" s="40" t="inlineStr">
         <is>
           <t>진행 중</t>
         </is>
       </c>
-      <c r="I52" s="39" t="n">
+      <c r="I53" s="41" t="n">
         <v>0.3</v>
       </c>
-      <c r="J52" s="8" t="inlineStr">
+      <c r="J53" s="8" t="inlineStr">
         <is>
           <t>PR #30 시연 순서</t>
         </is>
       </c>
-      <c r="K52" s="8" t="n"/>
+      <c r="K53" s="8" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K52"/>
-  <conditionalFormatting sqref="H5:H52">
+  <autoFilter ref="A4:K53"/>
+  <conditionalFormatting sqref="H5:H53">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"완료"</formula>
     </cfRule>
@@ -2868,7 +2921,7 @@
       <formula>"보류"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I52">
+  <conditionalFormatting sqref="I5:I53">
     <cfRule type="dataBar" priority="4">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -2878,10 +2931,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="H5:H52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"완료,진행 중,예정,보류"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E5:E53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"개발,디자인,공동"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2952,23 +3005,23 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A4,WBS!$H$5:$H$52,"&lt;&gt;")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A4,WBS!$H$5:$H$53,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C4" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A4,WBS!$H$5:$H$52,"완료")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A4,WBS!$H$5:$H$53,"완료")</f>
         <v/>
       </c>
       <c r="D4" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A4,WBS!$H$5:$H$52,"진행 중")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A4,WBS!$H$5:$H$53,"진행 중")</f>
         <v/>
       </c>
       <c r="E4" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A4,WBS!$H$5:$H$52,"예정")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A4,WBS!$H$5:$H$53,"예정")</f>
         <v/>
       </c>
       <c r="F4" s="12">
-        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$52,WBS!$B$5:$B$52,A4,WBS!$H$5:$H$52,"&lt;&gt;"),0)</f>
+        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$53,WBS!$B$5:$B$53,A4,WBS!$H$5:$H$53,"&lt;&gt;"),0)</f>
         <v/>
       </c>
     </row>
@@ -2979,23 +3032,23 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A5,WBS!$H$5:$H$52,"&lt;&gt;")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A5,WBS!$H$5:$H$53,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C5" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A5,WBS!$H$5:$H$52,"완료")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A5,WBS!$H$5:$H$53,"완료")</f>
         <v/>
       </c>
       <c r="D5" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A5,WBS!$H$5:$H$52,"진행 중")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A5,WBS!$H$5:$H$53,"진행 중")</f>
         <v/>
       </c>
       <c r="E5" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A5,WBS!$H$5:$H$52,"예정")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A5,WBS!$H$5:$H$53,"예정")</f>
         <v/>
       </c>
       <c r="F5" s="12">
-        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$52,WBS!$B$5:$B$52,A5,WBS!$H$5:$H$52,"&lt;&gt;"),0)</f>
+        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$53,WBS!$B$5:$B$53,A5,WBS!$H$5:$H$53,"&lt;&gt;"),0)</f>
         <v/>
       </c>
     </row>
@@ -3006,23 +3059,23 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A6,WBS!$H$5:$H$52,"&lt;&gt;")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A6,WBS!$H$5:$H$53,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C6" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A6,WBS!$H$5:$H$52,"완료")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A6,WBS!$H$5:$H$53,"완료")</f>
         <v/>
       </c>
       <c r="D6" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A6,WBS!$H$5:$H$52,"진행 중")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A6,WBS!$H$5:$H$53,"진행 중")</f>
         <v/>
       </c>
       <c r="E6" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A6,WBS!$H$5:$H$52,"예정")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A6,WBS!$H$5:$H$53,"예정")</f>
         <v/>
       </c>
       <c r="F6" s="12">
-        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$52,WBS!$B$5:$B$52,A6,WBS!$H$5:$H$52,"&lt;&gt;"),0)</f>
+        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$53,WBS!$B$5:$B$53,A6,WBS!$H$5:$H$53,"&lt;&gt;"),0)</f>
         <v/>
       </c>
     </row>
@@ -3033,23 +3086,23 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A7,WBS!$H$5:$H$52,"&lt;&gt;")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A7,WBS!$H$5:$H$53,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C7" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A7,WBS!$H$5:$H$52,"완료")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A7,WBS!$H$5:$H$53,"완료")</f>
         <v/>
       </c>
       <c r="D7" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A7,WBS!$H$5:$H$52,"진행 중")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A7,WBS!$H$5:$H$53,"진행 중")</f>
         <v/>
       </c>
       <c r="E7" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A7,WBS!$H$5:$H$52,"예정")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A7,WBS!$H$5:$H$53,"예정")</f>
         <v/>
       </c>
       <c r="F7" s="12">
-        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$52,WBS!$B$5:$B$52,A7,WBS!$H$5:$H$52,"&lt;&gt;"),0)</f>
+        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$53,WBS!$B$5:$B$53,A7,WBS!$H$5:$H$53,"&lt;&gt;"),0)</f>
         <v/>
       </c>
     </row>
@@ -3060,23 +3113,23 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A8,WBS!$H$5:$H$52,"&lt;&gt;")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A8,WBS!$H$5:$H$53,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C8" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A8,WBS!$H$5:$H$52,"완료")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A8,WBS!$H$5:$H$53,"완료")</f>
         <v/>
       </c>
       <c r="D8" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A8,WBS!$H$5:$H$52,"진행 중")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A8,WBS!$H$5:$H$53,"진행 중")</f>
         <v/>
       </c>
       <c r="E8" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A8,WBS!$H$5:$H$52,"예정")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A8,WBS!$H$5:$H$53,"예정")</f>
         <v/>
       </c>
       <c r="F8" s="12">
-        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$52,WBS!$B$5:$B$52,A8,WBS!$H$5:$H$52,"&lt;&gt;"),0)</f>
+        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$53,WBS!$B$5:$B$53,A8,WBS!$H$5:$H$53,"&lt;&gt;"),0)</f>
         <v/>
       </c>
     </row>
@@ -3087,23 +3140,23 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A9,WBS!$H$5:$H$52,"&lt;&gt;")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A9,WBS!$H$5:$H$53,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C9" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A9,WBS!$H$5:$H$52,"완료")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A9,WBS!$H$5:$H$53,"완료")</f>
         <v/>
       </c>
       <c r="D9" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A9,WBS!$H$5:$H$52,"진행 중")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A9,WBS!$H$5:$H$53,"진행 중")</f>
         <v/>
       </c>
       <c r="E9" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A9,WBS!$H$5:$H$52,"예정")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A9,WBS!$H$5:$H$53,"예정")</f>
         <v/>
       </c>
       <c r="F9" s="12">
-        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$52,WBS!$B$5:$B$52,A9,WBS!$H$5:$H$52,"&lt;&gt;"),0)</f>
+        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$53,WBS!$B$5:$B$53,A9,WBS!$H$5:$H$53,"&lt;&gt;"),0)</f>
         <v/>
       </c>
     </row>
@@ -3114,23 +3167,23 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A10,WBS!$H$5:$H$52,"&lt;&gt;")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A10,WBS!$H$5:$H$53,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C10" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A10,WBS!$H$5:$H$52,"완료")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A10,WBS!$H$5:$H$53,"완료")</f>
         <v/>
       </c>
       <c r="D10" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A10,WBS!$H$5:$H$52,"진행 중")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A10,WBS!$H$5:$H$53,"진행 중")</f>
         <v/>
       </c>
       <c r="E10" s="11">
-        <f>COUNTIFS(WBS!$B$5:$B$52,A10,WBS!$H$5:$H$52,"예정")</f>
+        <f>COUNTIFS(WBS!$B$5:$B$53,A10,WBS!$H$5:$H$53,"예정")</f>
         <v/>
       </c>
       <c r="F10" s="12">
-        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$52,WBS!$B$5:$B$52,A10,WBS!$H$5:$H$52,"&lt;&gt;"),0)</f>
+        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$53,WBS!$B$5:$B$53,A10,WBS!$H$5:$H$53,"&lt;&gt;"),0)</f>
         <v/>
       </c>
     </row>
@@ -3157,7 +3210,7 @@
         <v/>
       </c>
       <c r="F11" s="14">
-        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$52,WBS!$H$5:$H$52,"&lt;&gt;"),0)</f>
+        <f>IFERROR(AVERAGEIFS(WBS!$I$5:$I$53,WBS!$H$5:$H$53,"&lt;&gt;"),0)</f>
         <v/>
       </c>
     </row>

</xml_diff>